<commit_message>
feat(revenue-stream): add Total Car Care Treatments day/MTD to the Excel export
New total_car_care_treatments_daily precompute, recomputed alongside
Unique VIN VAS on every Service Info (GS/BP) upload: every TGLOSS-priced
job-code line billed (not deduped per RO), on an RO not closed by an
accessories-staff SA. Wires rows 97/98 of the Revenue Stream template to
the new report.ts fields, and strips the template's old "(w/o Mech Care)"
wording from those labels (a surgical edit to the xlsx's shared strings
only, verified byte-identical elsewhere) — this now counts every TGLOSS
treatment type, Mech Care included, at the user's request. October
backfilled; MTD totals confirmed against a prior manual check.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/revenue-stream-template.xlsx
+++ b/templates/revenue-stream-template.xlsx
@@ -546,13 +546,13 @@
     <t>Unique VIN VAS  for the  day</t>
   </si>
   <si>
-    <t>Total Car Care Treatments Target(w/o Mech Care)</t>
+    <t>Total Car Care Treatments Target</t>
   </si>
   <si>
-    <t>Total Car Care Treatments  for the  day(w/o Mech Care)</t>
+    <t>Total Car Care Treatments  for the  day</t>
   </si>
   <si>
-    <t>Achvmnt for the month(w/o Mech Care)</t>
+    <t>Achvmnt for the month</t>
   </si>
   <si>
     <t>TP-TP Target</t>

</xml_diff>